<commit_message>
feat: added original rows order
</commit_message>
<xml_diff>
--- a/testfile.xlsx
+++ b/testfile.xlsx
@@ -109,32 +109,32 @@
     <t>Differences</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Removed: functionality | Added: another func</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Yes</t>
+    <t>Removed: name | Added: surname</t>
   </si>
   <si>
     <t>Removed: Hello | Added: Hi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Removed: Hello,
+Some message content
+CTA: functionality</t>
   </si>
   <si>
     <t xml:space="preserve">Added: Hello,
 Some message content
 CTA: functionality</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed: Hello,
-Some message content
-CTA: functionality</t>
-  </si>
-  <si>
-    <t>Removed: functionality | Added: another func</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Removed: name | Added: surname</t>
   </si>
 </sst>
 </file>
@@ -734,39 +734,39 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" t="s">
         <v>26</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>27</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -774,19 +774,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
         <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s">
-        <v>27</v>
       </c>
       <c r="F4" t="s">
         <v>30</v>
@@ -794,19 +794,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
         <v>31</v>
@@ -814,39 +814,39 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
         <v>32</v>
-      </c>
-      <c r="F6" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
feat: handling rich text and filtering
</commit_message>
<xml_diff>
--- a/testfile.xlsx
+++ b/testfile.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520"/>
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="Old" state="visible" r:id="rId4"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="35">
   <si>
     <t>Type</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Colum 4</t>
+  </si>
+  <si>
+    <t>Filter</t>
   </si>
   <si>
     <t>First notification type</t>
@@ -45,7 +48,13 @@
 CTA: functionality</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>Second notification type</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
   <si>
     <t>Third notification type</t>
@@ -67,9 +76,43 @@
     <t>6th notification</t>
   </si>
   <si>
-    <t xml:space="preserve">Hello,
+    <r>
+      <t xml:space="preserve">Hello,
 Some message content
-CTA: another func</t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>CTA:</t>
+    </r>
+    <r>
+      <rPr>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>another func</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Hi,
@@ -109,19 +152,13 @@
     <t>Differences</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Removed: functionality | Added: another func</t>
   </si>
   <si>
-    <t>No</t>
+    <t>Removed: name | Added: surname</t>
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>Removed: name | Added: surname</t>
   </si>
   <si>
     <t>Removed: Hello | Added: Hi</t>
@@ -173,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -181,7 +218,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,14 +505,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="5" max="5" width="29.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -488,66 +531,84 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F2" s="1"/>
-    </row>
-    <row r="3" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" s="1"/>
-    </row>
-    <row r="4" ht="75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" ht="75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1"/>
-    </row>
-    <row r="5" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F5" s="1"/>
-    </row>
-    <row r="6" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" s="1"/>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -556,14 +617,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="5" max="5" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -582,66 +643,84 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F2" s="1"/>
-    </row>
-    <row r="3" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" s="1"/>
-    </row>
-    <row r="4" ht="75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" ht="75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F4" s="1"/>
-    </row>
-    <row r="5" ht="75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F5" s="1"/>
-    </row>
-    <row r="6" ht="60" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" s="1"/>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -664,7 +743,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -672,26 +751,26 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -701,155 +780,131 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="61" customWidth="1"/>
-    <col min="3" max="3" width="63" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="61" style="3" customWidth="1"/>
+    <col min="3" max="3" width="63" style="3" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>25</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>14</v>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C4" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
         <v>16</v>
       </c>
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3"/>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
+        <v>20</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>